<commit_message>
chore: update Sheets via scheduled runner
</commit_message>
<xml_diff>
--- a/Sheets/Adamantoise_Profits.xlsx
+++ b/Sheets/Adamantoise_Profits.xlsx
@@ -808,26 +808,23 @@
         <v>5470</v>
       </c>
       <c r="H4" t="n">
-        <v>475</v>
+        <v>500</v>
       </c>
       <c r="I4" t="n">
         <v>500</v>
       </c>
       <c r="J4" t="n">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>500</v>
       </c>
       <c r="L4" t="n">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
         <v>-386</v>
       </c>
-      <c r="N4" t="n">
-        <v>-678</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -860,22 +857,22 @@
         <v>5503</v>
       </c>
       <c r="H5" t="n">
-        <v>284.33334</v>
+        <v>411</v>
       </c>
       <c r="I5" t="n">
-        <v>204.5</v>
+        <v>400</v>
       </c>
       <c r="J5" t="n">
         <v>444</v>
       </c>
       <c r="K5" t="n">
-        <v>204.5</v>
+        <v>400</v>
       </c>
       <c r="L5" t="n">
         <v>444</v>
       </c>
       <c r="M5" t="n">
-        <v>-89.5</v>
+        <v>-285</v>
       </c>
       <c r="N5" t="n">
         <v>-674</v>
@@ -1056,25 +1053,22 @@
         <v>5487</v>
       </c>
       <c r="H9" t="n">
-        <v>352.83334</v>
+        <v>432.66666</v>
       </c>
       <c r="I9" t="n">
-        <v>379</v>
+        <v>432.66666</v>
       </c>
       <c r="J9" t="n">
-        <v>222</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>379</v>
+        <v>432.66666</v>
       </c>
       <c r="L9" t="n">
-        <v>222</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>-210</v>
-      </c>
-      <c r="N9" t="n">
-        <v>-560</v>
+        <v>-263.66666</v>
       </c>
     </row>
     <row r="10">
@@ -1399,22 +1393,22 @@
         <v>2146</v>
       </c>
       <c r="H16" t="n">
-        <v>4666.6665</v>
+        <v>4497.5</v>
       </c>
       <c r="I16" t="n">
-        <v>4000</v>
+        <v>3995</v>
       </c>
       <c r="J16" t="n">
         <v>5000</v>
       </c>
       <c r="K16" t="n">
-        <v>4000</v>
+        <v>3995</v>
       </c>
       <c r="L16" t="n">
         <v>5000</v>
       </c>
       <c r="M16" t="n">
-        <v>-3770</v>
+        <v>-3765</v>
       </c>
       <c r="N16" t="n">
         <v>-5460</v>
@@ -1500,25 +1494,22 @@
         <v>5471</v>
       </c>
       <c r="H18" t="n">
-        <v>1091.25</v>
+        <v>1201</v>
       </c>
       <c r="I18" t="n">
-        <v>1206.4286</v>
+        <v>1201</v>
       </c>
       <c r="J18" t="n">
-        <v>285</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1206.4286</v>
+        <v>1201</v>
       </c>
       <c r="L18" t="n">
-        <v>285</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>-922.4286</v>
-      </c>
-      <c r="N18" t="n">
-        <v>-853</v>
+        <v>-917</v>
       </c>
     </row>
     <row r="19">
@@ -2036,22 +2027,22 @@
         <v>4575</v>
       </c>
       <c r="H29" t="n">
-        <v>877</v>
+        <v>823.1667</v>
       </c>
       <c r="I29" t="n">
-        <v>569.5</v>
+        <v>646.3333</v>
       </c>
       <c r="J29" t="n">
         <v>1000</v>
       </c>
       <c r="K29" t="n">
-        <v>1708.5</v>
+        <v>1938.9999</v>
       </c>
       <c r="L29" t="n">
         <v>3000</v>
       </c>
       <c r="M29" t="n">
-        <v>-1427.5</v>
+        <v>-1657.9999</v>
       </c>
       <c r="N29" t="n">
         <v>-3562</v>
@@ -2477,23 +2468,26 @@
         <v>4599</v>
       </c>
       <c r="H38" t="n">
-        <v>266.33334</v>
+        <v>439.6</v>
       </c>
       <c r="I38" t="n">
         <v>266.33334</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1999</v>
       </c>
       <c r="K38" t="n">
         <v>799.0000200000001</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>5997</v>
       </c>
       <c r="M38" t="n">
         <v>-427.0000200000001</v>
       </c>
+      <c r="N38" t="n">
+        <v>-6741</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2578,25 +2572,25 @@
         <v>5505</v>
       </c>
       <c r="H40" t="n">
-        <v>146642.86</v>
+        <v>146571.42</v>
       </c>
       <c r="I40" t="n">
-        <v>3000000</v>
+        <v>1501000</v>
       </c>
       <c r="J40" t="n">
-        <v>3975</v>
+        <v>4000</v>
       </c>
       <c r="K40" t="n">
-        <v>3000000</v>
+        <v>1501000</v>
       </c>
       <c r="L40" t="n">
-        <v>3975</v>
+        <v>4000</v>
       </c>
       <c r="M40" t="n">
-        <v>-2999825</v>
+        <v>-1500825</v>
       </c>
       <c r="N40" t="n">
-        <v>-4325</v>
+        <v>-4350</v>
       </c>
     </row>
     <row r="41">
@@ -2731,25 +2725,25 @@
         <v>5472</v>
       </c>
       <c r="H43" t="n">
-        <v>7992</v>
+        <v>8225.083000000001</v>
       </c>
       <c r="I43" t="n">
-        <v>6665.8335</v>
+        <v>6133.3335</v>
       </c>
       <c r="J43" t="n">
-        <v>9128.714</v>
+        <v>10316.833</v>
       </c>
       <c r="K43" t="n">
-        <v>6665.8335</v>
+        <v>6133.3335</v>
       </c>
       <c r="L43" t="n">
-        <v>9128.714</v>
+        <v>10316.833</v>
       </c>
       <c r="M43" t="n">
-        <v>-6596.8335</v>
+        <v>-6064.3335</v>
       </c>
       <c r="N43" t="n">
-        <v>-9266.714</v>
+        <v>-10454.833</v>
       </c>
     </row>
     <row r="44">
@@ -3227,22 +3221,22 @@
         <v>5479</v>
       </c>
       <c r="H53" t="n">
-        <v>1404.6875</v>
+        <v>1325</v>
       </c>
       <c r="I53" t="n">
-        <v>660.0769</v>
+        <v>616.5</v>
       </c>
       <c r="J53" t="n">
         <v>4631.3335</v>
       </c>
       <c r="K53" t="n">
-        <v>660.0769</v>
+        <v>616.5</v>
       </c>
       <c r="L53" t="n">
         <v>4631.3335</v>
       </c>
       <c r="M53" t="n">
-        <v>-23.07690000000002</v>
+        <v>20.5</v>
       </c>
       <c r="N53" t="n">
         <v>-5905.3335</v>
@@ -3279,19 +3273,22 @@
         <v>2174</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L54" t="n">
         <v>0</v>
+      </c>
+      <c r="M54" t="n">
+        <v>-514</v>
       </c>
     </row>
     <row r="55">
@@ -3668,25 +3665,25 @@
         <v>27781</v>
       </c>
       <c r="H62" t="n">
-        <v>9119.5</v>
+        <v>8682.25</v>
       </c>
       <c r="I62" t="n">
-        <v>8357.857</v>
+        <v>7938</v>
       </c>
       <c r="J62" t="n">
-        <v>10896.667</v>
+        <v>10170.75</v>
       </c>
       <c r="K62" t="n">
-        <v>8357.857</v>
+        <v>7938</v>
       </c>
       <c r="L62" t="n">
-        <v>10896.667</v>
+        <v>10170.75</v>
       </c>
       <c r="M62" t="n">
-        <v>-7733.857</v>
+        <v>-7314</v>
       </c>
       <c r="N62" t="n">
-        <v>-12144.667</v>
+        <v>-11418.75</v>
       </c>
     </row>
     <row r="63">
@@ -3818,25 +3815,25 @@
         <v>27781</v>
       </c>
       <c r="H65" t="n">
-        <v>9119.5</v>
+        <v>8682.25</v>
       </c>
       <c r="I65" t="n">
-        <v>8357.857</v>
+        <v>7938</v>
       </c>
       <c r="J65" t="n">
-        <v>10896.667</v>
+        <v>10170.75</v>
       </c>
       <c r="K65" t="n">
-        <v>41789.285</v>
+        <v>39690</v>
       </c>
       <c r="L65" t="n">
-        <v>54483.335</v>
+        <v>50853.75</v>
       </c>
       <c r="M65" t="n">
-        <v>-38669.285</v>
+        <v>-36570</v>
       </c>
       <c r="N65" t="n">
-        <v>-60723.335</v>
+        <v>-57093.75</v>
       </c>
     </row>
     <row r="66">
@@ -4908,25 +4905,25 @@
         <v>10651</v>
       </c>
       <c r="H87" t="n">
-        <v>94531.25</v>
+        <v>96897.14</v>
       </c>
       <c r="I87" t="n">
         <v>77489</v>
       </c>
       <c r="J87" t="n">
-        <v>96965.86</v>
+        <v>100131.836</v>
       </c>
       <c r="K87" t="n">
         <v>77489</v>
       </c>
       <c r="L87" t="n">
-        <v>96965.86</v>
+        <v>100131.836</v>
       </c>
       <c r="M87" t="n">
         <v>-76241</v>
       </c>
       <c r="N87" t="n">
-        <v>-99461.86</v>
+        <v>-102627.836</v>
       </c>
     </row>
     <row r="88">
@@ -5061,25 +5058,25 @@
         <v>10651</v>
       </c>
       <c r="H90" t="n">
-        <v>94531.25</v>
+        <v>96897.14</v>
       </c>
       <c r="I90" t="n">
         <v>77489</v>
       </c>
       <c r="J90" t="n">
-        <v>96965.86</v>
+        <v>100131.836</v>
       </c>
       <c r="K90" t="n">
         <v>232467</v>
       </c>
       <c r="L90" t="n">
-        <v>290897.58</v>
+        <v>300395.508</v>
       </c>
       <c r="M90" t="n">
         <v>-226227</v>
       </c>
       <c r="N90" t="n">
-        <v>-303377.58</v>
+        <v>-312875.508</v>
       </c>
     </row>
     <row r="91">
@@ -5459,22 +5456,22 @@
         <v>36237</v>
       </c>
       <c r="H98" t="n">
-        <v>7103.5884</v>
+        <v>6730.24</v>
       </c>
       <c r="I98" t="n">
-        <v>7157.7334</v>
+        <v>6733.087</v>
       </c>
       <c r="J98" t="n">
         <v>6697.5</v>
       </c>
       <c r="K98" t="n">
-        <v>7157.7334</v>
+        <v>6733.087</v>
       </c>
       <c r="L98" t="n">
         <v>6697.5</v>
       </c>
       <c r="M98" t="n">
-        <v>-5659.7334</v>
+        <v>-5235.087</v>
       </c>
       <c r="N98" t="n">
         <v>-9693.5</v>
@@ -5563,25 +5560,25 @@
         <v>19906</v>
       </c>
       <c r="H100" t="n">
-        <v>2397.1538</v>
+        <v>2454.96</v>
       </c>
       <c r="I100" t="n">
         <v>1563</v>
       </c>
       <c r="J100" t="n">
-        <v>2918.5</v>
+        <v>3049.6</v>
       </c>
       <c r="K100" t="n">
         <v>1563</v>
       </c>
       <c r="L100" t="n">
-        <v>2918.5</v>
+        <v>3049.6</v>
       </c>
       <c r="M100" t="n">
         <v>-1022</v>
       </c>
       <c r="N100" t="n">
-        <v>-4000.5</v>
+        <v>-4131.6</v>
       </c>
     </row>
     <row r="101">
@@ -5915,25 +5912,25 @@
         <v>27766</v>
       </c>
       <c r="H107" t="n">
-        <v>2590.9285</v>
+        <v>3133.4285</v>
       </c>
       <c r="I107" t="n">
-        <v>2298.182</v>
+        <v>2800.4375</v>
       </c>
       <c r="J107" t="n">
-        <v>3664.3333</v>
+        <v>4199</v>
       </c>
       <c r="K107" t="n">
-        <v>2298.182</v>
+        <v>2800.4375</v>
       </c>
       <c r="L107" t="n">
-        <v>3664.3333</v>
+        <v>4199</v>
       </c>
       <c r="M107" t="n">
-        <v>-378.1819999999998</v>
+        <v>-880.4375</v>
       </c>
       <c r="N107" t="n">
-        <v>-7504.3333</v>
+        <v>-8039</v>
       </c>
     </row>
     <row r="108">
@@ -6368,22 +6365,22 @@
         <v>71453096</v>
       </c>
       <c r="I116" t="n">
-        <v>125039780</v>
+        <v>166718340</v>
       </c>
       <c r="J116" t="n">
-        <v>4199</v>
+        <v>4174.25</v>
       </c>
       <c r="K116" t="n">
-        <v>125039780</v>
+        <v>166718340</v>
       </c>
       <c r="L116" t="n">
-        <v>4199</v>
+        <v>4174.25</v>
       </c>
       <c r="M116" t="n">
-        <v>-125036338</v>
+        <v>-166714898</v>
       </c>
       <c r="N116" t="n">
-        <v>-11083</v>
+        <v>-11058.25</v>
       </c>
     </row>
     <row r="117">
@@ -6668,22 +6665,22 @@
         <v>36237</v>
       </c>
       <c r="H122" t="n">
-        <v>7103.5884</v>
+        <v>6730.24</v>
       </c>
       <c r="I122" t="n">
-        <v>7157.7334</v>
+        <v>6733.087</v>
       </c>
       <c r="J122" t="n">
         <v>6697.5</v>
       </c>
       <c r="K122" t="n">
-        <v>21473.2002</v>
+        <v>20199.261</v>
       </c>
       <c r="L122" t="n">
         <v>20092.5</v>
       </c>
       <c r="M122" t="n">
-        <v>-19023.2002</v>
+        <v>-17749.261</v>
       </c>
       <c r="N122" t="n">
         <v>-24992.5</v>
@@ -7017,25 +7014,25 @@
         <v>36115</v>
       </c>
       <c r="H129" t="n">
-        <v>1966.9333</v>
+        <v>1919.4667</v>
       </c>
       <c r="I129" t="n">
         <v>1381</v>
       </c>
       <c r="J129" t="n">
-        <v>2845.8333</v>
+        <v>2727.1667</v>
       </c>
       <c r="K129" t="n">
         <v>4143</v>
       </c>
       <c r="L129" t="n">
-        <v>8537.499899999999</v>
+        <v>8181.500100000001</v>
       </c>
       <c r="M129" t="n">
         <v>857</v>
       </c>
       <c r="N129" t="n">
-        <v>-18537.4999</v>
+        <v>-18181.5001</v>
       </c>
     </row>
     <row r="130">
@@ -7170,22 +7167,22 @@
         <v>44049</v>
       </c>
       <c r="H132" t="n">
-        <v>3018.8125</v>
+        <v>2461.3333</v>
       </c>
       <c r="I132" t="n">
-        <v>3018.8125</v>
+        <v>2461.3333</v>
       </c>
       <c r="J132" t="n">
         <v>0</v>
       </c>
       <c r="K132" t="n">
-        <v>9056.4375</v>
+        <v>7383.999899999999</v>
       </c>
       <c r="L132" t="n">
         <v>0</v>
       </c>
       <c r="M132" t="n">
-        <v>-6526.4375</v>
+        <v>-4853.999899999999</v>
       </c>
     </row>
     <row r="133">
@@ -7219,22 +7216,22 @@
         <v>41856</v>
       </c>
       <c r="H133" t="n">
-        <v>108331.664</v>
+        <v>109997.5</v>
       </c>
       <c r="I133" t="n">
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>108331.664</v>
+        <v>109997.5</v>
       </c>
       <c r="K133" t="n">
         <v>0</v>
       </c>
       <c r="L133" t="n">
-        <v>108331.664</v>
+        <v>109997.5</v>
       </c>
       <c r="N133" t="n">
-        <v>-118451.664</v>
+        <v>-120117.5</v>
       </c>
     </row>
     <row r="134">
@@ -7317,22 +7314,22 @@
         <v>44047</v>
       </c>
       <c r="H135" t="n">
-        <v>446.34616</v>
+        <v>433.33334</v>
       </c>
       <c r="I135" t="n">
-        <v>457.52</v>
+        <v>443.57693</v>
       </c>
       <c r="J135" t="n">
         <v>167</v>
       </c>
       <c r="K135" t="n">
-        <v>4117.68</v>
+        <v>3992.19237</v>
       </c>
       <c r="L135" t="n">
         <v>1503</v>
       </c>
       <c r="M135" t="n">
-        <v>-1582.68</v>
+        <v>-1457.19237</v>
       </c>
       <c r="N135" t="n">
         <v>-6573</v>
@@ -7418,25 +7415,25 @@
         <v>44013</v>
       </c>
       <c r="H137" t="n">
-        <v>1558.8</v>
+        <v>1543.4546</v>
       </c>
       <c r="I137" t="n">
         <v>1417</v>
       </c>
       <c r="J137" t="n">
-        <v>1619.5714</v>
+        <v>1590.875</v>
       </c>
       <c r="K137" t="n">
         <v>4251</v>
       </c>
       <c r="L137" t="n">
-        <v>4858.7142</v>
+        <v>4772.625</v>
       </c>
       <c r="M137" t="n">
         <v>-1701</v>
       </c>
       <c r="N137" t="n">
-        <v>-9958.7142</v>
+        <v>-9872.625</v>
       </c>
     </row>
     <row r="138">
@@ -7470,25 +7467,25 @@
         <v>44169</v>
       </c>
       <c r="H138" t="n">
-        <v>3554.43</v>
+        <v>3511.42</v>
       </c>
       <c r="I138" t="n">
-        <v>2030.875</v>
+        <v>1714.7</v>
       </c>
       <c r="J138" t="n">
-        <v>3686.913</v>
+        <v>3711.0557</v>
       </c>
       <c r="K138" t="n">
-        <v>6092.625</v>
+        <v>5144.1</v>
       </c>
       <c r="L138" t="n">
-        <v>11060.739</v>
+        <v>11133.1671</v>
       </c>
       <c r="M138" t="n">
-        <v>-952.625</v>
+        <v>-4.100000000000364</v>
       </c>
       <c r="N138" t="n">
-        <v>-21340.739</v>
+        <v>-21413.1671</v>
       </c>
     </row>
     <row r="139">
@@ -7617,25 +7614,25 @@
         <v>44161</v>
       </c>
       <c r="H141" t="n">
-        <v>4202.636</v>
+        <v>4168.3145</v>
       </c>
       <c r="I141" t="n">
-        <v>4147.7036</v>
+        <v>4178.2856</v>
       </c>
       <c r="J141" t="n">
-        <v>4449.8335</v>
+        <v>4128.4287</v>
       </c>
       <c r="K141" t="n">
-        <v>12443.1108</v>
+        <v>12534.8568</v>
       </c>
       <c r="L141" t="n">
-        <v>13349.5005</v>
+        <v>12385.2861</v>
       </c>
       <c r="M141" t="n">
-        <v>-7263.110799999999</v>
+        <v>-7354.856800000001</v>
       </c>
       <c r="N141" t="n">
-        <v>-23709.5005</v>
+        <v>-22745.2861</v>
       </c>
     </row>
   </sheetData>
@@ -7758,25 +7755,25 @@
         <v>27713</v>
       </c>
       <c r="H2" t="n">
-        <v>1673.9445</v>
+        <v>1444.7894</v>
       </c>
       <c r="I2" t="n">
-        <v>1130.7858</v>
+        <v>1034.4375</v>
       </c>
       <c r="J2" t="n">
-        <v>3575</v>
+        <v>3633.3333</v>
       </c>
       <c r="K2" t="n">
-        <v>1130.7858</v>
+        <v>1034.4375</v>
       </c>
       <c r="L2" t="n">
-        <v>3575</v>
+        <v>3633.3333</v>
       </c>
       <c r="M2" t="n">
-        <v>-1017.7858</v>
+        <v>-921.4375</v>
       </c>
       <c r="N2" t="n">
-        <v>-3801</v>
+        <v>-3859.3333</v>
       </c>
     </row>
     <row r="3">
@@ -9231,22 +9228,22 @@
         <v>44147</v>
       </c>
       <c r="H32" t="n">
-        <v>28275980</v>
+        <v>27550956</v>
       </c>
       <c r="I32" t="n">
-        <v>36273310</v>
+        <v>35022510</v>
       </c>
       <c r="J32" t="n">
         <v>5883451</v>
       </c>
       <c r="K32" t="n">
-        <v>36273310</v>
+        <v>35022510</v>
       </c>
       <c r="L32" t="n">
         <v>5883451</v>
       </c>
       <c r="M32" t="n">
-        <v>-36273023</v>
+        <v>-35022223</v>
       </c>
       <c r="N32" t="n">
         <v>-5884025</v>
@@ -10637,25 +10634,25 @@
         <v>43999</v>
       </c>
       <c r="H61" t="n">
-        <v>2913.742</v>
+        <v>2768.597</v>
       </c>
       <c r="I61" t="n">
-        <v>2381.5122</v>
+        <v>2247.568</v>
       </c>
       <c r="J61" t="n">
-        <v>3952.8572</v>
+        <v>3765.348</v>
       </c>
       <c r="K61" t="n">
-        <v>2381.5122</v>
+        <v>2247.568</v>
       </c>
       <c r="L61" t="n">
-        <v>3952.8572</v>
+        <v>3765.348</v>
       </c>
       <c r="M61" t="n">
-        <v>-2169.5122</v>
+        <v>-2035.568</v>
       </c>
       <c r="N61" t="n">
-        <v>-4376.8572</v>
+        <v>-4189.348</v>
       </c>
     </row>
     <row r="62">
@@ -11259,22 +11256,22 @@
         <v>44000</v>
       </c>
       <c r="H74" t="n">
-        <v>1789.1818</v>
+        <v>1698.1041</v>
       </c>
       <c r="I74" t="n">
-        <v>1762.4872</v>
+        <v>1663.3024</v>
       </c>
       <c r="J74" t="n">
         <v>1997.4</v>
       </c>
       <c r="K74" t="n">
-        <v>1762.4872</v>
+        <v>1663.3024</v>
       </c>
       <c r="L74" t="n">
         <v>1997.4</v>
       </c>
       <c r="M74" t="n">
-        <v>-888.4872</v>
+        <v>-789.3024</v>
       </c>
       <c r="N74" t="n">
         <v>-3745.4</v>
@@ -11406,22 +11403,22 @@
         <v>44000</v>
       </c>
       <c r="H77" t="n">
-        <v>1789.1818</v>
+        <v>1698.1041</v>
       </c>
       <c r="I77" t="n">
-        <v>1762.4872</v>
+        <v>1663.3024</v>
       </c>
       <c r="J77" t="n">
         <v>1997.4</v>
       </c>
       <c r="K77" t="n">
-        <v>8812.436</v>
+        <v>8316.512000000001</v>
       </c>
       <c r="L77" t="n">
         <v>9987</v>
       </c>
       <c r="M77" t="n">
-        <v>-4444.436</v>
+        <v>-3948.512000000001</v>
       </c>
       <c r="N77" t="n">
         <v>-18723</v>
@@ -12135,19 +12132,22 @@
         <v>18050</v>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>121499</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
       </c>
       <c r="J92" t="n">
-        <v>0</v>
+        <v>121499</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
       </c>
       <c r="L92" t="n">
-        <v>0</v>
+        <v>121499</v>
+      </c>
+      <c r="N92" t="n">
+        <v>-126491</v>
       </c>
     </row>
     <row r="93">
@@ -13011,25 +13011,25 @@
         <v>27708</v>
       </c>
       <c r="H110" t="n">
-        <v>1302.9062</v>
+        <v>1401.138</v>
       </c>
       <c r="I110" t="n">
-        <v>551.8421</v>
+        <v>559.8889</v>
       </c>
       <c r="J110" t="n">
-        <v>2400.6155</v>
+        <v>2777.7273</v>
       </c>
       <c r="K110" t="n">
-        <v>551.8421</v>
+        <v>559.8889</v>
       </c>
       <c r="L110" t="n">
-        <v>2400.6155</v>
+        <v>2777.7273</v>
       </c>
       <c r="M110" t="n">
-        <v>1493.1579</v>
+        <v>1485.1111</v>
       </c>
       <c r="N110" t="n">
-        <v>-6490.6155</v>
+        <v>-6867.7273</v>
       </c>
     </row>
     <row r="111">
@@ -13305,25 +13305,25 @@
         <v>27713</v>
       </c>
       <c r="H116" t="n">
-        <v>1673.9445</v>
+        <v>1444.7894</v>
       </c>
       <c r="I116" t="n">
-        <v>1130.7858</v>
+        <v>1034.4375</v>
       </c>
       <c r="J116" t="n">
-        <v>3575</v>
+        <v>3633.3333</v>
       </c>
       <c r="K116" t="n">
-        <v>1130.7858</v>
+        <v>1034.4375</v>
       </c>
       <c r="L116" t="n">
-        <v>3575</v>
+        <v>3633.3333</v>
       </c>
       <c r="M116" t="n">
-        <v>1163.2142</v>
+        <v>1259.5625</v>
       </c>
       <c r="N116" t="n">
-        <v>-8163</v>
+        <v>-8221.3333</v>
       </c>
     </row>
     <row r="117">
@@ -13599,25 +13599,25 @@
         <v>36168</v>
       </c>
       <c r="H122" t="n">
-        <v>2008.6727</v>
+        <v>1910.7273</v>
       </c>
       <c r="I122" t="n">
-        <v>1428.279</v>
+        <v>1398.2954</v>
       </c>
       <c r="J122" t="n">
-        <v>4088.4167</v>
+        <v>3960.4546</v>
       </c>
       <c r="K122" t="n">
-        <v>4284.837</v>
+        <v>4194.8862</v>
       </c>
       <c r="L122" t="n">
-        <v>12265.2501</v>
+        <v>11881.3638</v>
       </c>
       <c r="M122" t="n">
-        <v>-1834.837</v>
+        <v>-1744.8862</v>
       </c>
       <c r="N122" t="n">
-        <v>-17165.2501</v>
+        <v>-16781.3638</v>
       </c>
     </row>
     <row r="123">
@@ -14086,25 +14086,25 @@
         <v>43997</v>
       </c>
       <c r="H132" t="n">
-        <v>1632.4717</v>
+        <v>1551.4036</v>
       </c>
       <c r="I132" t="n">
-        <v>1520.0197</v>
+        <v>1460</v>
       </c>
       <c r="J132" t="n">
-        <v>4500</v>
+        <v>3196.6667</v>
       </c>
       <c r="K132" t="n">
-        <v>4560.0591</v>
+        <v>4380</v>
       </c>
       <c r="L132" t="n">
-        <v>13500</v>
+        <v>9590.000100000001</v>
       </c>
       <c r="M132" t="n">
-        <v>-2030.0591</v>
+        <v>-1850</v>
       </c>
       <c r="N132" t="n">
-        <v>-18560</v>
+        <v>-14650.0001</v>
       </c>
     </row>
     <row r="133">
@@ -14233,22 +14233,19 @@
         <v>42016</v>
       </c>
       <c r="H135" t="n">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="I135" t="n">
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="K135" t="n">
         <v>0</v>
       </c>
       <c r="L135" t="n">
-        <v>80000</v>
-      </c>
-      <c r="N135" t="n">
-        <v>-90140</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -14282,25 +14279,25 @@
         <v>43999</v>
       </c>
       <c r="H136" t="n">
-        <v>2913.742</v>
+        <v>2768.597</v>
       </c>
       <c r="I136" t="n">
-        <v>2381.5122</v>
+        <v>2247.568</v>
       </c>
       <c r="J136" t="n">
-        <v>3952.8572</v>
+        <v>3765.348</v>
       </c>
       <c r="K136" t="n">
-        <v>7144.5366</v>
+        <v>6742.704000000001</v>
       </c>
       <c r="L136" t="n">
-        <v>11858.5716</v>
+        <v>11296.044</v>
       </c>
       <c r="M136" t="n">
-        <v>-4594.5366</v>
+        <v>-4192.704000000001</v>
       </c>
       <c r="N136" t="n">
-        <v>-16958.5716</v>
+        <v>-16396.044</v>
       </c>
     </row>
     <row r="137">
@@ -14714,25 +14711,25 @@
         <v>27713</v>
       </c>
       <c r="H3" t="n">
-        <v>1673.9445</v>
+        <v>1444.7894</v>
       </c>
       <c r="I3" t="n">
-        <v>1130.7858</v>
+        <v>1034.4375</v>
       </c>
       <c r="J3" t="n">
-        <v>3575</v>
+        <v>3633.3333</v>
       </c>
       <c r="K3" t="n">
-        <v>1130.7858</v>
+        <v>1034.4375</v>
       </c>
       <c r="L3" t="n">
-        <v>3575</v>
+        <v>3633.3333</v>
       </c>
       <c r="M3" t="n">
-        <v>-1016.7858</v>
+        <v>-920.4375</v>
       </c>
       <c r="N3" t="n">
-        <v>-3803</v>
+        <v>-3861.3333</v>
       </c>
     </row>
     <row r="4">
@@ -15538,25 +15535,25 @@
         <v>14149</v>
       </c>
       <c r="H20" t="n">
-        <v>2318.625</v>
+        <v>3300</v>
       </c>
       <c r="I20" t="n">
-        <v>2299.5</v>
+        <v>3924.5</v>
       </c>
       <c r="J20" t="n">
-        <v>2337.75</v>
+        <v>2883.6667</v>
       </c>
       <c r="K20" t="n">
-        <v>2299.5</v>
+        <v>3924.5</v>
       </c>
       <c r="L20" t="n">
-        <v>2337.75</v>
+        <v>2883.6667</v>
       </c>
       <c r="M20" t="n">
-        <v>-2052.5</v>
+        <v>-3677.5</v>
       </c>
       <c r="N20" t="n">
-        <v>-2831.75</v>
+        <v>-3377.6667</v>
       </c>
     </row>
     <row r="21">
@@ -15636,22 +15633,25 @@
         <v>5092</v>
       </c>
       <c r="H22" t="n">
-        <v>91</v>
+        <v>86.25</v>
       </c>
       <c r="I22" t="n">
-        <v>91</v>
+        <v>91.666664</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="K22" t="n">
-        <v>91</v>
+        <v>91.666664</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="M22" t="n">
-        <v>82</v>
+        <v>81.333336</v>
+      </c>
+      <c r="N22" t="n">
+        <v>-416</v>
       </c>
     </row>
     <row r="23">
@@ -15777,22 +15777,25 @@
         <v>2370</v>
       </c>
       <c r="H25" t="n">
-        <v>4000</v>
+        <v>3999.6667</v>
       </c>
       <c r="I25" t="n">
-        <v>4000</v>
+        <v>3499.5</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="K25" t="n">
-        <v>4000</v>
+        <v>3499.5</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="M25" t="n">
-        <v>-3765</v>
+        <v>-3264.5</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-5470</v>
       </c>
     </row>
     <row r="26">
@@ -16365,25 +16368,22 @@
         <v>2485</v>
       </c>
       <c r="H37" t="n">
-        <v>1681.5</v>
+        <v>2249.5</v>
       </c>
       <c r="I37" t="n">
-        <v>2272.25</v>
+        <v>2249.5</v>
       </c>
       <c r="J37" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>2272.25</v>
+        <v>2249.5</v>
       </c>
       <c r="L37" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-2135.25</v>
-      </c>
-      <c r="N37" t="n">
-        <v>-774</v>
+        <v>-2112.5</v>
       </c>
     </row>
     <row r="38">
@@ -18757,25 +18757,25 @@
         <v>12526</v>
       </c>
       <c r="H86" t="n">
-        <v>4911.5</v>
+        <v>4610.375</v>
       </c>
       <c r="I86" t="n">
-        <v>4295</v>
+        <v>4220.75</v>
       </c>
       <c r="J86" t="n">
-        <v>5117</v>
+        <v>5000</v>
       </c>
       <c r="K86" t="n">
-        <v>4295</v>
+        <v>4220.75</v>
       </c>
       <c r="L86" t="n">
-        <v>5117</v>
+        <v>5000</v>
       </c>
       <c r="M86" t="n">
-        <v>-3172</v>
+        <v>-3097.75</v>
       </c>
       <c r="N86" t="n">
-        <v>-7363</v>
+        <v>-7246</v>
       </c>
     </row>
     <row r="87">
@@ -18901,25 +18901,25 @@
         <v>12526</v>
       </c>
       <c r="H89" t="n">
-        <v>4911.5</v>
+        <v>4610.375</v>
       </c>
       <c r="I89" t="n">
-        <v>4295</v>
+        <v>4220.75</v>
       </c>
       <c r="J89" t="n">
-        <v>5117</v>
+        <v>5000</v>
       </c>
       <c r="K89" t="n">
-        <v>21475</v>
+        <v>21103.75</v>
       </c>
       <c r="L89" t="n">
-        <v>25585</v>
+        <v>25000</v>
       </c>
       <c r="M89" t="n">
-        <v>-15859</v>
+        <v>-15487.75</v>
       </c>
       <c r="N89" t="n">
-        <v>-36817</v>
+        <v>-36232</v>
       </c>
     </row>
     <row r="90">
@@ -19143,22 +19143,22 @@
         <v>19939</v>
       </c>
       <c r="H94" t="n">
-        <v>674.125</v>
+        <v>622.13336</v>
       </c>
       <c r="I94" t="n">
-        <v>608.5294</v>
+        <v>556.9487</v>
       </c>
       <c r="J94" t="n">
         <v>1045.8334</v>
       </c>
       <c r="K94" t="n">
-        <v>608.5294</v>
+        <v>556.9487</v>
       </c>
       <c r="L94" t="n">
         <v>1045.8334</v>
       </c>
       <c r="M94" t="n">
-        <v>-157.5294</v>
+        <v>-105.9487</v>
       </c>
       <c r="N94" t="n">
         <v>-1947.8334</v>
@@ -19394,22 +19394,22 @@
         <v>19943</v>
       </c>
       <c r="H99" t="n">
-        <v>4548.625</v>
+        <v>3965.5</v>
       </c>
       <c r="I99" t="n">
-        <v>4731.5</v>
+        <v>3958.6</v>
       </c>
       <c r="J99" t="n">
         <v>4000</v>
       </c>
       <c r="K99" t="n">
-        <v>4731.5</v>
+        <v>3958.6</v>
       </c>
       <c r="L99" t="n">
         <v>4000</v>
       </c>
       <c r="M99" t="n">
-        <v>-3233.5</v>
+        <v>-2460.6</v>
       </c>
       <c r="N99" t="n">
         <v>-6996</v>
@@ -19691,22 +19691,22 @@
         <v>19947</v>
       </c>
       <c r="H105" t="n">
-        <v>1977.6666</v>
+        <v>1926.742</v>
       </c>
       <c r="I105" t="n">
-        <v>1699.7826</v>
+        <v>1645.5834</v>
       </c>
       <c r="J105" t="n">
         <v>2890.7144</v>
       </c>
       <c r="K105" t="n">
-        <v>1699.7826</v>
+        <v>1645.5834</v>
       </c>
       <c r="L105" t="n">
         <v>2890.7144</v>
       </c>
       <c r="M105" t="n">
-        <v>47.2174</v>
+        <v>101.4166</v>
       </c>
       <c r="N105" t="n">
         <v>-6384.7144</v>
@@ -19792,22 +19792,22 @@
         <v>27706</v>
       </c>
       <c r="H107" t="n">
-        <v>1773.4722</v>
+        <v>1757.9429</v>
       </c>
       <c r="I107" t="n">
-        <v>1720.6</v>
+        <v>1695.75</v>
       </c>
       <c r="J107" t="n">
         <v>1893.6364</v>
       </c>
       <c r="K107" t="n">
-        <v>1720.6</v>
+        <v>1695.75</v>
       </c>
       <c r="L107" t="n">
         <v>1893.6364</v>
       </c>
       <c r="M107" t="n">
-        <v>199.4000000000001</v>
+        <v>224.25</v>
       </c>
       <c r="N107" t="n">
         <v>-5733.6364</v>
@@ -20714,22 +20714,22 @@
         <v>34398</v>
       </c>
       <c r="H126" t="n">
-        <v>206000</v>
+        <v>160000</v>
       </c>
       <c r="I126" t="n">
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>206000</v>
+        <v>160000</v>
       </c>
       <c r="K126" t="n">
         <v>0</v>
       </c>
       <c r="L126" t="n">
-        <v>206000</v>
+        <v>160000</v>
       </c>
       <c r="N126" t="n">
-        <v>-215880</v>
+        <v>-169880</v>
       </c>
     </row>
     <row r="127">
@@ -20999,22 +20999,22 @@
         <v>41855</v>
       </c>
       <c r="H132" t="n">
-        <v>129330</v>
+        <v>134995</v>
       </c>
       <c r="I132" t="n">
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>129330</v>
+        <v>134995</v>
       </c>
       <c r="K132" t="n">
         <v>0</v>
       </c>
       <c r="L132" t="n">
-        <v>129330</v>
+        <v>134995</v>
       </c>
       <c r="N132" t="n">
-        <v>-139450</v>
+        <v>-145115</v>
       </c>
     </row>
     <row r="133">
@@ -21097,25 +21097,25 @@
         <v>43998</v>
       </c>
       <c r="H134" t="n">
-        <v>1390597.4</v>
+        <v>1308709</v>
       </c>
       <c r="I134" t="n">
-        <v>1551597.1</v>
+        <v>1419556.6</v>
       </c>
       <c r="J134" t="n">
-        <v>5998.8</v>
+        <v>6248.5</v>
       </c>
       <c r="K134" t="n">
-        <v>4654791.300000001</v>
+        <v>4258669.800000001</v>
       </c>
       <c r="L134" t="n">
-        <v>17996.4</v>
+        <v>18745.5</v>
       </c>
       <c r="M134" t="n">
-        <v>-4652256.300000001</v>
+        <v>-4256134.800000001</v>
       </c>
       <c r="N134" t="n">
-        <v>-23066.4</v>
+        <v>-23815.5</v>
       </c>
     </row>
     <row r="135">
@@ -21428,22 +21428,22 @@
         <v>43278</v>
       </c>
       <c r="H141" t="n">
-        <v>155640</v>
+        <v>188250</v>
       </c>
       <c r="I141" t="n">
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>155640</v>
+        <v>188250</v>
       </c>
       <c r="K141" t="n">
         <v>0</v>
       </c>
       <c r="L141" t="n">
-        <v>155640</v>
+        <v>188250</v>
       </c>
       <c r="N141" t="n">
-        <v>-166000</v>
+        <v>-198610</v>
       </c>
     </row>
   </sheetData>
@@ -21713,25 +21713,25 @@
         <v>1893</v>
       </c>
       <c r="H5" t="n">
-        <v>2747.25</v>
+        <v>2486.3333</v>
       </c>
       <c r="I5" t="n">
         <v>4135.8</v>
       </c>
       <c r="J5" t="n">
-        <v>433</v>
+        <v>424.5</v>
       </c>
       <c r="K5" t="n">
         <v>4135.8</v>
       </c>
       <c r="L5" t="n">
-        <v>433</v>
+        <v>424.5</v>
       </c>
       <c r="M5" t="n">
         <v>-4023.8</v>
       </c>
       <c r="N5" t="n">
-        <v>-657</v>
+        <v>-648.5</v>
       </c>
     </row>
     <row r="6">
@@ -21814,22 +21814,22 @@
         <v>5361</v>
       </c>
       <c r="H7" t="n">
-        <v>70.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="I7" t="n">
-        <v>70.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>70.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>42.40000000000001</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="8">
@@ -22243,22 +22243,19 @@
         <v>27691</v>
       </c>
       <c r="H16" t="n">
-        <v>724</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>724</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>724</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>-437</v>
       </c>
     </row>
     <row r="17">
@@ -22987,25 +22984,25 @@
         <v>44023</v>
       </c>
       <c r="H31" t="n">
-        <v>2179.606</v>
+        <v>2109.2856</v>
       </c>
       <c r="I31" t="n">
-        <v>1997.5</v>
+        <v>1854.8572</v>
       </c>
       <c r="J31" t="n">
-        <v>2220.074</v>
+        <v>2172.8928</v>
       </c>
       <c r="K31" t="n">
-        <v>1997.5</v>
+        <v>1854.8572</v>
       </c>
       <c r="L31" t="n">
-        <v>2220.074</v>
+        <v>2172.8928</v>
       </c>
       <c r="M31" t="n">
-        <v>-1702.5</v>
+        <v>-1559.8572</v>
       </c>
       <c r="N31" t="n">
-        <v>-2810.074</v>
+        <v>-2762.8928</v>
       </c>
     </row>
     <row r="32">
@@ -23140,25 +23137,25 @@
         <v>44023</v>
       </c>
       <c r="H34" t="n">
-        <v>2179.606</v>
+        <v>2109.2856</v>
       </c>
       <c r="I34" t="n">
-        <v>1997.5</v>
+        <v>1854.8572</v>
       </c>
       <c r="J34" t="n">
-        <v>2220.074</v>
+        <v>2172.8928</v>
       </c>
       <c r="K34" t="n">
-        <v>1997.5</v>
+        <v>1854.8572</v>
       </c>
       <c r="L34" t="n">
-        <v>2220.074</v>
+        <v>2172.8928</v>
       </c>
       <c r="M34" t="n">
-        <v>-1795.5</v>
+        <v>-1652.8572</v>
       </c>
       <c r="N34" t="n">
-        <v>-2624.074</v>
+        <v>-2576.8928</v>
       </c>
     </row>
     <row r="35">
@@ -24074,22 +24071,22 @@
         <v>25632</v>
       </c>
       <c r="H53" t="n">
-        <v>24995</v>
+        <v>25000</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>24995</v>
+        <v>25000</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
       </c>
       <c r="L53" t="n">
-        <v>24995</v>
+        <v>25000</v>
       </c>
       <c r="N53" t="n">
-        <v>-26209</v>
+        <v>-26214</v>
       </c>
     </row>
     <row r="54">
@@ -25667,25 +25664,25 @@
         <v>12584</v>
       </c>
       <c r="H86" t="n">
-        <v>10449.889</v>
+        <v>9935.655000000001</v>
       </c>
       <c r="I86" t="n">
-        <v>12242.429</v>
+        <v>10564.765</v>
       </c>
       <c r="J86" t="n">
-        <v>8519.462</v>
+        <v>9044.416999999999</v>
       </c>
       <c r="K86" t="n">
-        <v>12242.429</v>
+        <v>10564.765</v>
       </c>
       <c r="L86" t="n">
-        <v>8519.462</v>
+        <v>9044.416999999999</v>
       </c>
       <c r="M86" t="n">
-        <v>-11119.429</v>
+        <v>-9441.764999999999</v>
       </c>
       <c r="N86" t="n">
-        <v>-10765.462</v>
+        <v>-11290.417</v>
       </c>
     </row>
     <row r="87">
@@ -25817,25 +25814,25 @@
         <v>12584</v>
       </c>
       <c r="H89" t="n">
-        <v>10449.889</v>
+        <v>9935.655000000001</v>
       </c>
       <c r="I89" t="n">
-        <v>12242.429</v>
+        <v>10564.765</v>
       </c>
       <c r="J89" t="n">
-        <v>8519.462</v>
+        <v>9044.416999999999</v>
       </c>
       <c r="K89" t="n">
-        <v>61212.145</v>
+        <v>52823.825</v>
       </c>
       <c r="L89" t="n">
-        <v>42597.31</v>
+        <v>45222.085</v>
       </c>
       <c r="M89" t="n">
-        <v>-55596.145</v>
+        <v>-47207.825</v>
       </c>
       <c r="N89" t="n">
-        <v>-53829.31</v>
+        <v>-56454.085</v>
       </c>
     </row>
     <row r="90">
@@ -26567,22 +26564,22 @@
         <v>19749</v>
       </c>
       <c r="H104" t="n">
-        <v>64918.332</v>
+        <v>64915</v>
       </c>
       <c r="I104" t="n">
         <v>0</v>
       </c>
       <c r="J104" t="n">
-        <v>64918.332</v>
+        <v>64915</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
       </c>
       <c r="L104" t="n">
-        <v>64918.332</v>
+        <v>64915</v>
       </c>
       <c r="N104" t="n">
-        <v>-70160.33199999999</v>
+        <v>-70157</v>
       </c>
     </row>
     <row r="105">
@@ -26717,25 +26714,25 @@
         <v>27689</v>
       </c>
       <c r="H107" t="n">
-        <v>979.3333</v>
+        <v>1049.25</v>
       </c>
       <c r="I107" t="n">
         <v>1648</v>
       </c>
       <c r="J107" t="n">
-        <v>788.2857</v>
+        <v>849.6667</v>
       </c>
       <c r="K107" t="n">
         <v>1648</v>
       </c>
       <c r="L107" t="n">
-        <v>788.2857</v>
+        <v>849.6667</v>
       </c>
       <c r="M107" t="n">
         <v>272</v>
       </c>
       <c r="N107" t="n">
-        <v>-4628.2857</v>
+        <v>-4689.6667</v>
       </c>
     </row>
     <row r="108">
@@ -26916,19 +26913,22 @@
         <v>25792</v>
       </c>
       <c r="H111" t="n">
-        <v>0</v>
+        <v>155000</v>
       </c>
       <c r="I111" t="n">
         <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>155000</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
       </c>
       <c r="L111" t="n">
-        <v>0</v>
+        <v>155000</v>
+      </c>
+      <c r="N111" t="n">
+        <v>-163180</v>
       </c>
     </row>
     <row r="112">
@@ -27011,22 +27011,19 @@
         <v>27691</v>
       </c>
       <c r="H113" t="n">
-        <v>724</v>
+        <v>0</v>
       </c>
       <c r="I113" t="n">
-        <v>724</v>
+        <v>0</v>
       </c>
       <c r="J113" t="n">
         <v>0</v>
       </c>
       <c r="K113" t="n">
-        <v>724</v>
+        <v>0</v>
       </c>
       <c r="L113" t="n">
         <v>0</v>
-      </c>
-      <c r="M113" t="n">
-        <v>1446</v>
       </c>
     </row>
     <row r="114">
@@ -27446,25 +27443,25 @@
         <v>36196</v>
       </c>
       <c r="H122" t="n">
-        <v>4037.5293</v>
+        <v>3957.8948</v>
       </c>
       <c r="I122" t="n">
-        <v>3588.9</v>
+        <v>3700.0908</v>
       </c>
       <c r="J122" t="n">
-        <v>4678.4287</v>
+        <v>4312.375</v>
       </c>
       <c r="K122" t="n">
-        <v>10766.7</v>
+        <v>11100.2724</v>
       </c>
       <c r="L122" t="n">
-        <v>14035.2861</v>
+        <v>12937.125</v>
       </c>
       <c r="M122" t="n">
-        <v>-8316.700000000001</v>
+        <v>-8650.2724</v>
       </c>
       <c r="N122" t="n">
-        <v>-18935.2861</v>
+        <v>-17837.125</v>
       </c>
     </row>
     <row r="123">
@@ -27933,25 +27930,25 @@
         <v>44019</v>
       </c>
       <c r="H132" t="n">
-        <v>2610.3</v>
+        <v>2420.8076</v>
       </c>
       <c r="I132" t="n">
-        <v>2059.875</v>
+        <v>2044</v>
       </c>
       <c r="J132" t="n">
-        <v>4812</v>
+        <v>4003.4</v>
       </c>
       <c r="K132" t="n">
-        <v>6179.625</v>
+        <v>6132</v>
       </c>
       <c r="L132" t="n">
-        <v>14436</v>
+        <v>12010.2</v>
       </c>
       <c r="M132" t="n">
-        <v>-3649.625</v>
+        <v>-3602</v>
       </c>
       <c r="N132" t="n">
-        <v>-19496</v>
+        <v>-17070.2</v>
       </c>
     </row>
     <row r="133">
@@ -28034,22 +28031,22 @@
         <v>44020</v>
       </c>
       <c r="H134" t="n">
-        <v>1632.1111</v>
+        <v>1588.5172</v>
       </c>
       <c r="I134" t="n">
-        <v>1482.72</v>
+        <v>1446.963</v>
       </c>
       <c r="J134" t="n">
         <v>3499.5</v>
       </c>
       <c r="K134" t="n">
-        <v>4448.16</v>
+        <v>4340.889</v>
       </c>
       <c r="L134" t="n">
         <v>10498.5</v>
       </c>
       <c r="M134" t="n">
-        <v>-1913.16</v>
+        <v>-1805.889</v>
       </c>
       <c r="N134" t="n">
         <v>-15568.5</v>
@@ -28383,25 +28380,25 @@
         <v>43345</v>
       </c>
       <c r="H141" t="n">
-        <v>1049987</v>
+        <v>894663.8</v>
       </c>
       <c r="I141" t="n">
         <v>59999</v>
       </c>
       <c r="J141" t="n">
-        <v>1297484</v>
+        <v>1061596.8</v>
       </c>
       <c r="K141" t="n">
         <v>59999</v>
       </c>
       <c r="L141" t="n">
-        <v>1297484</v>
+        <v>1061596.8</v>
       </c>
       <c r="M141" t="n">
         <v>-54819</v>
       </c>
       <c r="N141" t="n">
-        <v>-1307844</v>
+        <v>-1071956.8</v>
       </c>
     </row>
   </sheetData>
@@ -29133,22 +29130,22 @@
         <v>12886</v>
       </c>
       <c r="H14" t="n">
-        <v>1292.3334</v>
+        <v>826.1</v>
       </c>
       <c r="I14" t="n">
-        <v>1292.3334</v>
+        <v>826.1</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>3877.0002</v>
+        <v>2478.3</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>-3704.0002</v>
+        <v>-2305.3</v>
       </c>
     </row>
     <row r="15">
@@ -30752,22 +30749,19 @@
         <v>4701</v>
       </c>
       <c r="H46" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
-      </c>
-      <c r="M46" t="n">
-        <v>-119</v>
       </c>
     </row>
     <row r="47">
@@ -31539,22 +31533,19 @@
         <v>12845</v>
       </c>
       <c r="H62" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>336</v>
+        <v>0</v>
       </c>
       <c r="L62" t="n">
         <v>0</v>
-      </c>
-      <c r="M62" t="n">
-        <v>350</v>
       </c>
     </row>
     <row r="63">
@@ -31588,22 +31579,22 @@
         <v>12866</v>
       </c>
       <c r="H63" t="n">
-        <v>12</v>
+        <v>5000</v>
       </c>
       <c r="I63" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="K63" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
-      </c>
-      <c r="M63" t="n">
-        <v>713</v>
+        <v>15000</v>
+      </c>
+      <c r="N63" t="n">
+        <v>-16498</v>
       </c>
     </row>
     <row r="64">
@@ -31683,22 +31674,19 @@
         <v>12845</v>
       </c>
       <c r="H65" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>1008</v>
+        <v>0</v>
       </c>
       <c r="L65" t="n">
         <v>0</v>
-      </c>
-      <c r="M65" t="n">
-        <v>2424</v>
       </c>
     </row>
     <row r="66">
@@ -31732,22 +31720,22 @@
         <v>12866</v>
       </c>
       <c r="H66" t="n">
-        <v>12</v>
+        <v>5000</v>
       </c>
       <c r="I66" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="K66" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
-      </c>
-      <c r="M66" t="n">
-        <v>3636</v>
+        <v>45000</v>
+      </c>
+      <c r="N66" t="n">
+        <v>-52488</v>
       </c>
     </row>
     <row r="67">
@@ -31827,25 +31815,25 @@
         <v>12895</v>
       </c>
       <c r="H68" t="n">
-        <v>1753.0869</v>
+        <v>1744.5217</v>
       </c>
       <c r="I68" t="n">
-        <v>1425</v>
+        <v>1377.6666</v>
       </c>
       <c r="J68" t="n">
-        <v>1928.0667</v>
+        <v>1980.3572</v>
       </c>
       <c r="K68" t="n">
-        <v>4275</v>
+        <v>4132.9998</v>
       </c>
       <c r="L68" t="n">
-        <v>5784.2001</v>
+        <v>5941.071599999999</v>
       </c>
       <c r="M68" t="n">
-        <v>-3464</v>
+        <v>-3321.9998</v>
       </c>
       <c r="N68" t="n">
-        <v>-7406.2001</v>
+        <v>-7563.071599999999</v>
       </c>
     </row>
     <row r="69">
@@ -31980,25 +31968,25 @@
         <v>12895</v>
       </c>
       <c r="H71" t="n">
-        <v>1753.0869</v>
+        <v>1744.5217</v>
       </c>
       <c r="I71" t="n">
-        <v>1425</v>
+        <v>1377.6666</v>
       </c>
       <c r="J71" t="n">
-        <v>1928.0667</v>
+        <v>1980.3572</v>
       </c>
       <c r="K71" t="n">
-        <v>12825</v>
+        <v>12398.9994</v>
       </c>
       <c r="L71" t="n">
-        <v>17352.6003</v>
+        <v>17823.2148</v>
       </c>
       <c r="M71" t="n">
-        <v>-8769</v>
+        <v>-8342.999400000001</v>
       </c>
       <c r="N71" t="n">
-        <v>-25464.6003</v>
+        <v>-25935.2148</v>
       </c>
     </row>
     <row r="72">
@@ -32421,25 +32409,25 @@
         <v>12890</v>
       </c>
       <c r="H80" t="n">
-        <v>3374.75</v>
+        <v>4699.6</v>
       </c>
       <c r="I80" t="n">
         <v>1166.3334</v>
       </c>
       <c r="J80" t="n">
-        <v>10000</v>
+        <v>9999.5</v>
       </c>
       <c r="K80" t="n">
         <v>3499.0002</v>
       </c>
       <c r="L80" t="n">
-        <v>30000</v>
+        <v>29998.5</v>
       </c>
       <c r="M80" t="n">
         <v>-2563.0002</v>
       </c>
       <c r="N80" t="n">
-        <v>-31872</v>
+        <v>-31870.5</v>
       </c>
     </row>
     <row r="81">
@@ -32571,25 +32559,25 @@
         <v>12890</v>
       </c>
       <c r="H83" t="n">
-        <v>3374.75</v>
+        <v>4699.6</v>
       </c>
       <c r="I83" t="n">
         <v>1166.3334</v>
       </c>
       <c r="J83" t="n">
-        <v>10000</v>
+        <v>9999.5</v>
       </c>
       <c r="K83" t="n">
         <v>10497.0006</v>
       </c>
       <c r="L83" t="n">
-        <v>90000</v>
+        <v>89995.5</v>
       </c>
       <c r="M83" t="n">
         <v>-5817.000599999999</v>
       </c>
       <c r="N83" t="n">
-        <v>-99360</v>
+        <v>-99355.5</v>
       </c>
     </row>
     <row r="84">
@@ -33009,25 +32997,25 @@
         <v>19841</v>
       </c>
       <c r="H92" t="n">
-        <v>817.8333</v>
+        <v>758.7692</v>
       </c>
       <c r="I92" t="n">
         <v>560</v>
       </c>
       <c r="J92" t="n">
-        <v>946.75</v>
+        <v>847.1111</v>
       </c>
       <c r="K92" t="n">
         <v>1680</v>
       </c>
       <c r="L92" t="n">
-        <v>2840.25</v>
+        <v>2541.3333</v>
       </c>
       <c r="M92" t="n">
         <v>-432</v>
       </c>
       <c r="N92" t="n">
-        <v>-5336.25</v>
+        <v>-5037.3333</v>
       </c>
     </row>
     <row r="93">
@@ -33747,25 +33735,25 @@
         <v>27838</v>
       </c>
       <c r="H107" t="n">
-        <v>1215.3846</v>
+        <v>1185.7693</v>
       </c>
       <c r="I107" t="n">
         <v>1174.5555</v>
       </c>
       <c r="J107" t="n">
-        <v>1237</v>
+        <v>1191.7059</v>
       </c>
       <c r="K107" t="n">
         <v>3523.6665</v>
       </c>
       <c r="L107" t="n">
-        <v>3711</v>
+        <v>3575.1177</v>
       </c>
       <c r="M107" t="n">
         <v>-1603.6665</v>
       </c>
       <c r="N107" t="n">
-        <v>-7551</v>
+        <v>-7415.1177</v>
       </c>
     </row>
     <row r="108">
@@ -34050,25 +34038,25 @@
         <v>27843</v>
       </c>
       <c r="H113" t="n">
-        <v>2198.0715</v>
+        <v>2014.75</v>
       </c>
       <c r="I113" t="n">
         <v>2401.25</v>
       </c>
       <c r="J113" t="n">
-        <v>1927.1666</v>
+        <v>1628.25</v>
       </c>
       <c r="K113" t="n">
         <v>7203.75</v>
       </c>
       <c r="L113" t="n">
-        <v>5781.4998</v>
+        <v>4884.75</v>
       </c>
       <c r="M113" t="n">
         <v>-5033.75</v>
       </c>
       <c r="N113" t="n">
-        <v>-10121.4998</v>
+        <v>-9224.75</v>
       </c>
     </row>
     <row r="114">
@@ -34965,25 +34953,25 @@
         <v>36060</v>
       </c>
       <c r="H131" t="n">
-        <v>2150.2307</v>
+        <v>2512.111</v>
       </c>
       <c r="I131" t="n">
-        <v>2504</v>
+        <v>2479</v>
       </c>
       <c r="J131" t="n">
-        <v>2044.1</v>
+        <v>2545.2222</v>
       </c>
       <c r="K131" t="n">
-        <v>7512</v>
+        <v>7437</v>
       </c>
       <c r="L131" t="n">
-        <v>6132.299999999999</v>
+        <v>7635.6666</v>
       </c>
       <c r="M131" t="n">
-        <v>-2472</v>
+        <v>-2397</v>
       </c>
       <c r="N131" t="n">
-        <v>-16212.3</v>
+        <v>-17715.6666</v>
       </c>
     </row>
     <row r="132">
@@ -35268,25 +35256,25 @@
         <v>44088</v>
       </c>
       <c r="H137" t="n">
-        <v>2468</v>
+        <v>10129.23</v>
       </c>
       <c r="I137" t="n">
-        <v>1960</v>
+        <v>1964.4445</v>
       </c>
       <c r="J137" t="n">
-        <v>4500</v>
+        <v>28500</v>
       </c>
       <c r="K137" t="n">
-        <v>5880</v>
+        <v>5893.333500000001</v>
       </c>
       <c r="L137" t="n">
-        <v>13500</v>
+        <v>85500</v>
       </c>
       <c r="M137" t="n">
-        <v>-780</v>
+        <v>-793.3335000000006</v>
       </c>
       <c r="N137" t="n">
-        <v>-23700</v>
+        <v>-95700</v>
       </c>
     </row>
     <row r="138">
@@ -35421,22 +35409,22 @@
         <v>44097</v>
       </c>
       <c r="H140" t="n">
-        <v>2372.4443</v>
+        <v>2304.7273</v>
       </c>
       <c r="I140" t="n">
-        <v>1117.3334</v>
+        <v>1470.4</v>
       </c>
       <c r="J140" t="n">
         <v>3000</v>
       </c>
       <c r="K140" t="n">
-        <v>3352.0002</v>
+        <v>4411.200000000001</v>
       </c>
       <c r="L140" t="n">
         <v>9000</v>
       </c>
       <c r="M140" t="n">
-        <v>1827.9998</v>
+        <v>768.7999999999993</v>
       </c>
       <c r="N140" t="n">
         <v>-19360</v>
@@ -35859,22 +35847,22 @@
         <v>4197</v>
       </c>
       <c r="H7" t="n">
-        <v>6667367.5</v>
+        <v>10001000</v>
       </c>
       <c r="I7" t="n">
-        <v>6667367.5</v>
+        <v>10001000</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>6667367.5</v>
+        <v>10001000</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>-6667255.5</v>
+        <v>-10000888</v>
       </c>
     </row>
     <row r="8">
@@ -35908,22 +35896,22 @@
         <v>4197</v>
       </c>
       <c r="H8" t="n">
-        <v>6667367.5</v>
+        <v>10001000</v>
       </c>
       <c r="I8" t="n">
-        <v>6667367.5</v>
+        <v>10001000</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>6667367.5</v>
+        <v>10001000</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>-6667228.5</v>
+        <v>-10000861</v>
       </c>
     </row>
     <row r="9">
@@ -38297,22 +38285,25 @@
         <v>2876</v>
       </c>
       <c r="H57" t="n">
-        <v>28000</v>
+        <v>28999.5</v>
       </c>
       <c r="I57" t="n">
-        <v>28000</v>
+        <v>27999</v>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="K57" t="n">
-        <v>28000</v>
+        <v>27999</v>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="M57" t="n">
-        <v>-27180</v>
+        <v>-27179</v>
+      </c>
+      <c r="N57" t="n">
+        <v>-31640</v>
       </c>
     </row>
     <row r="58">
@@ -38536,25 +38527,25 @@
         <v>11983</v>
       </c>
       <c r="H62" t="n">
-        <v>52905</v>
+        <v>52820</v>
       </c>
       <c r="I62" t="n">
-        <v>46000</v>
+        <v>45945</v>
       </c>
       <c r="J62" t="n">
-        <v>59810</v>
+        <v>59695</v>
       </c>
       <c r="K62" t="n">
-        <v>46000</v>
+        <v>45945</v>
       </c>
       <c r="L62" t="n">
-        <v>59810</v>
+        <v>59695</v>
       </c>
       <c r="M62" t="n">
-        <v>-45314</v>
+        <v>-45259</v>
       </c>
       <c r="N62" t="n">
-        <v>-61182</v>
+        <v>-61067</v>
       </c>
     </row>
     <row r="63">
@@ -38686,25 +38677,25 @@
         <v>11983</v>
       </c>
       <c r="H65" t="n">
-        <v>52905</v>
+        <v>52820</v>
       </c>
       <c r="I65" t="n">
-        <v>46000</v>
+        <v>45945</v>
       </c>
       <c r="J65" t="n">
-        <v>59810</v>
+        <v>59695</v>
       </c>
       <c r="K65" t="n">
-        <v>138000</v>
+        <v>137835</v>
       </c>
       <c r="L65" t="n">
-        <v>179430</v>
+        <v>179085</v>
       </c>
       <c r="M65" t="n">
-        <v>-134568</v>
+        <v>-134403</v>
       </c>
       <c r="N65" t="n">
-        <v>-186294</v>
+        <v>-185949</v>
       </c>
     </row>
     <row r="66">
@@ -38931,25 +38922,25 @@
         <v>14146</v>
       </c>
       <c r="H70" t="n">
-        <v>27153.77</v>
+        <v>31272.727</v>
       </c>
       <c r="I70" t="n">
         <v>299000</v>
       </c>
       <c r="J70" t="n">
-        <v>4499.9165</v>
+        <v>4500</v>
       </c>
       <c r="K70" t="n">
         <v>299000</v>
       </c>
       <c r="L70" t="n">
-        <v>4499.9165</v>
+        <v>4500</v>
       </c>
       <c r="M70" t="n">
         <v>-298730</v>
       </c>
       <c r="N70" t="n">
-        <v>-5039.9165</v>
+        <v>-5040</v>
       </c>
     </row>
     <row r="71">
@@ -39078,25 +39069,25 @@
         <v>14146</v>
       </c>
       <c r="H73" t="n">
-        <v>27153.77</v>
+        <v>31272.727</v>
       </c>
       <c r="I73" t="n">
         <v>299000</v>
       </c>
       <c r="J73" t="n">
-        <v>4499.9165</v>
+        <v>4500</v>
       </c>
       <c r="K73" t="n">
         <v>299000</v>
       </c>
       <c r="L73" t="n">
-        <v>4499.9165</v>
+        <v>4500</v>
       </c>
       <c r="M73" t="n">
         <v>-298064</v>
       </c>
       <c r="N73" t="n">
-        <v>-6371.9165</v>
+        <v>-6372</v>
       </c>
     </row>
     <row r="74">
@@ -39406,22 +39397,22 @@
         <v>12521</v>
       </c>
       <c r="H80" t="n">
-        <v>3635.6</v>
+        <v>3363</v>
       </c>
       <c r="I80" t="n">
-        <v>3100</v>
+        <v>2733.3333</v>
       </c>
       <c r="J80" t="n">
         <v>3992.6667</v>
       </c>
       <c r="K80" t="n">
-        <v>3100</v>
+        <v>2733.3333</v>
       </c>
       <c r="L80" t="n">
         <v>3992.6667</v>
       </c>
       <c r="M80" t="n">
-        <v>-2102</v>
+        <v>-1735.3333</v>
       </c>
       <c r="N80" t="n">
         <v>-5988.6667</v>
@@ -39553,22 +39544,22 @@
         <v>12521</v>
       </c>
       <c r="H83" t="n">
-        <v>3635.6</v>
+        <v>3363</v>
       </c>
       <c r="I83" t="n">
-        <v>3100</v>
+        <v>2733.3333</v>
       </c>
       <c r="J83" t="n">
         <v>3992.6667</v>
       </c>
       <c r="K83" t="n">
-        <v>15500</v>
+        <v>13666.6665</v>
       </c>
       <c r="L83" t="n">
         <v>19963.3335</v>
       </c>
       <c r="M83" t="n">
-        <v>-10508</v>
+        <v>-8674.666499999999</v>
       </c>
       <c r="N83" t="n">
         <v>-29947.3335</v>
@@ -40080,22 +40071,22 @@
         <v>19511</v>
       </c>
       <c r="H94" t="n">
-        <v>84716.42999999999</v>
+        <v>77074</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
       </c>
       <c r="J94" t="n">
-        <v>84716.42999999999</v>
+        <v>77074</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
       </c>
       <c r="L94" t="n">
-        <v>84716.42999999999</v>
+        <v>77074</v>
       </c>
       <c r="N94" t="n">
-        <v>-86068.42999999999</v>
+        <v>-78426</v>
       </c>
     </row>
     <row r="95">
@@ -40472,25 +40463,25 @@
         <v>36169</v>
       </c>
       <c r="H102" t="n">
-        <v>1447.0416</v>
+        <v>1447</v>
       </c>
       <c r="I102" t="n">
         <v>1368.2858</v>
       </c>
       <c r="J102" t="n">
-        <v>1998.3334</v>
+        <v>1998</v>
       </c>
       <c r="K102" t="n">
         <v>1368.2858</v>
       </c>
       <c r="L102" t="n">
-        <v>1998.3334</v>
+        <v>1998</v>
       </c>
       <c r="M102" t="n">
         <v>253.7141999999999</v>
       </c>
       <c r="N102" t="n">
-        <v>-5242.3334</v>
+        <v>-5242</v>
       </c>
     </row>
     <row r="103">
@@ -41014,22 +41005,22 @@
         <v>27710</v>
       </c>
       <c r="H113" t="n">
-        <v>15725.826</v>
+        <v>15108.5</v>
       </c>
       <c r="I113" t="n">
-        <v>2014.5714</v>
+        <v>1940.9333</v>
       </c>
       <c r="J113" t="n">
         <v>37054.445</v>
       </c>
       <c r="K113" t="n">
-        <v>2014.5714</v>
+        <v>1940.9333</v>
       </c>
       <c r="L113" t="n">
         <v>37054.445</v>
       </c>
       <c r="M113" t="n">
-        <v>155.4286</v>
+        <v>229.0667000000001</v>
       </c>
       <c r="N113" t="n">
         <v>-41394.445</v>
@@ -41455,22 +41446,22 @@
         <v>2733.65</v>
       </c>
       <c r="I122" t="n">
-        <v>2903.1333</v>
+        <v>3058.5715</v>
       </c>
       <c r="J122" t="n">
-        <v>2225.2</v>
+        <v>1975.5</v>
       </c>
       <c r="K122" t="n">
-        <v>8709.3999</v>
+        <v>9175.7145</v>
       </c>
       <c r="L122" t="n">
-        <v>6675.599999999999</v>
+        <v>5926.5</v>
       </c>
       <c r="M122" t="n">
-        <v>-6259.3999</v>
+        <v>-6725.7145</v>
       </c>
       <c r="N122" t="n">
-        <v>-11575.6</v>
+        <v>-10826.5</v>
       </c>
     </row>
     <row r="123">
@@ -41654,25 +41645,25 @@
         <v>36184</v>
       </c>
       <c r="H126" t="n">
-        <v>3160.7896</v>
+        <v>2651.8845</v>
       </c>
       <c r="I126" t="n">
-        <v>2711.875</v>
+        <v>2462.182</v>
       </c>
       <c r="J126" t="n">
-        <v>3487.2727</v>
+        <v>2791</v>
       </c>
       <c r="K126" t="n">
-        <v>8135.625</v>
+        <v>7386.545999999999</v>
       </c>
       <c r="L126" t="n">
-        <v>10461.8181</v>
+        <v>8373</v>
       </c>
       <c r="M126" t="n">
-        <v>-5665.625</v>
+        <v>-4916.545999999999</v>
       </c>
       <c r="N126" t="n">
-        <v>-15401.8181</v>
+        <v>-13313</v>
       </c>
     </row>
     <row r="127">
@@ -41948,22 +41939,22 @@
         <v>44008</v>
       </c>
       <c r="H132" t="n">
-        <v>2313.762</v>
+        <v>2199.0881</v>
       </c>
       <c r="I132" t="n">
-        <v>1850.102</v>
+        <v>1748.6296</v>
       </c>
       <c r="J132" t="n">
         <v>3936.5715</v>
       </c>
       <c r="K132" t="n">
-        <v>5550.306</v>
+        <v>5245.8888</v>
       </c>
       <c r="L132" t="n">
         <v>11809.7145</v>
       </c>
       <c r="M132" t="n">
-        <v>-3020.306</v>
+        <v>-2715.8888</v>
       </c>
       <c r="N132" t="n">
         <v>-16869.7145</v>
@@ -42527,22 +42518,22 @@
         <v>2631</v>
       </c>
       <c r="H2" t="n">
-        <v>1318609.6</v>
+        <v>1376364.6</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1318609.6</v>
+        <v>1376364.6</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>1318609.6</v>
+        <v>1376364.6</v>
       </c>
       <c r="N2" t="n">
-        <v>-1318833.6</v>
+        <v>-1376588.6</v>
       </c>
     </row>
     <row r="3">
@@ -42775,25 +42766,25 @@
         <v>36249</v>
       </c>
       <c r="H7" t="n">
-        <v>6124.875</v>
+        <v>5760.3</v>
       </c>
       <c r="I7" t="n">
-        <v>4599</v>
+        <v>4932.3335</v>
       </c>
       <c r="J7" t="n">
-        <v>8668</v>
+        <v>7002.25</v>
       </c>
       <c r="K7" t="n">
-        <v>4599</v>
+        <v>4932.3335</v>
       </c>
       <c r="L7" t="n">
-        <v>8668</v>
+        <v>7002.25</v>
       </c>
       <c r="M7" t="n">
-        <v>-4487</v>
+        <v>-4820.3335</v>
       </c>
       <c r="N7" t="n">
-        <v>-8892</v>
+        <v>-7226.25</v>
       </c>
     </row>
     <row r="8">
@@ -43412,25 +43403,22 @@
         <v>4308</v>
       </c>
       <c r="H20" t="n">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="I20" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="J20" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="L20" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-774</v>
-      </c>
-      <c r="N20" t="n">
-        <v>-5452</v>
+        <v>-1274</v>
       </c>
     </row>
     <row r="21">
@@ -43464,22 +43452,22 @@
         <v>2672</v>
       </c>
       <c r="H21" t="n">
-        <v>10201.2</v>
+        <v>12001.5</v>
       </c>
       <c r="I21" t="n">
-        <v>11501.5</v>
+        <v>14335.333</v>
       </c>
       <c r="J21" t="n">
         <v>5000</v>
       </c>
       <c r="K21" t="n">
-        <v>11501.5</v>
+        <v>14335.333</v>
       </c>
       <c r="L21" t="n">
         <v>5000</v>
       </c>
       <c r="M21" t="n">
-        <v>-11327.5</v>
+        <v>-14161.333</v>
       </c>
       <c r="N21" t="n">
         <v>-5348</v>
@@ -43516,25 +43504,25 @@
         <v>5277</v>
       </c>
       <c r="H22" t="n">
-        <v>2307.52</v>
+        <v>2320.3333</v>
       </c>
       <c r="I22" t="n">
         <v>2186.5386</v>
       </c>
       <c r="J22" t="n">
-        <v>2438.5833</v>
+        <v>2478.4546</v>
       </c>
       <c r="K22" t="n">
         <v>2186.5386</v>
       </c>
       <c r="L22" t="n">
-        <v>2438.5833</v>
+        <v>2478.4546</v>
       </c>
       <c r="M22" t="n">
         <v>-1891.5386</v>
       </c>
       <c r="N22" t="n">
-        <v>-3028.5833</v>
+        <v>-3068.4546</v>
       </c>
     </row>
     <row r="23">
@@ -43614,22 +43602,22 @@
         <v>3774</v>
       </c>
       <c r="H24" t="n">
-        <v>14486</v>
+        <v>14856</v>
       </c>
       <c r="I24" t="n">
-        <v>14486</v>
+        <v>14856</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>14486</v>
+        <v>14856</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>-14143</v>
+        <v>-14513</v>
       </c>
     </row>
     <row r="25">
@@ -43761,25 +43749,25 @@
         <v>5277</v>
       </c>
       <c r="H27" t="n">
-        <v>2307.52</v>
+        <v>2320.3333</v>
       </c>
       <c r="I27" t="n">
         <v>2186.5386</v>
       </c>
       <c r="J27" t="n">
-        <v>2438.5833</v>
+        <v>2478.4546</v>
       </c>
       <c r="K27" t="n">
         <v>2186.5386</v>
       </c>
       <c r="L27" t="n">
-        <v>2438.5833</v>
+        <v>2478.4546</v>
       </c>
       <c r="M27" t="n">
         <v>-2079.5386</v>
       </c>
       <c r="N27" t="n">
-        <v>-2652.5833</v>
+        <v>-2692.4546</v>
       </c>
     </row>
     <row r="28">
@@ -44401,25 +44389,25 @@
         <v>36248</v>
       </c>
       <c r="H40" t="n">
-        <v>47621410</v>
+        <v>37039016</v>
       </c>
       <c r="I40" t="n">
-        <v>66668470</v>
+        <v>41668390</v>
       </c>
       <c r="J40" t="n">
-        <v>3752.5</v>
+        <v>4005</v>
       </c>
       <c r="K40" t="n">
-        <v>66668470</v>
+        <v>41668390</v>
       </c>
       <c r="L40" t="n">
-        <v>3752.5</v>
+        <v>4005</v>
       </c>
       <c r="M40" t="n">
-        <v>-66668334</v>
+        <v>-41668254</v>
       </c>
       <c r="N40" t="n">
-        <v>-4024.5</v>
+        <v>-4277</v>
       </c>
     </row>
     <row r="41">
@@ -44505,25 +44493,25 @@
         <v>4333</v>
       </c>
       <c r="H42" t="n">
-        <v>20951</v>
+        <v>40272.555</v>
       </c>
       <c r="I42" t="n">
-        <v>6412.5</v>
+        <v>6262.5</v>
       </c>
       <c r="J42" t="n">
-        <v>50028</v>
+        <v>49989.715</v>
       </c>
       <c r="K42" t="n">
-        <v>6412.5</v>
+        <v>6262.5</v>
       </c>
       <c r="L42" t="n">
-        <v>50028</v>
+        <v>49989.715</v>
       </c>
       <c r="M42" t="n">
-        <v>-5849.5</v>
+        <v>-5699.5</v>
       </c>
       <c r="N42" t="n">
-        <v>-51154</v>
+        <v>-51115.715</v>
       </c>
     </row>
     <row r="43">
@@ -44701,25 +44689,25 @@
         <v>5282</v>
       </c>
       <c r="H46" t="n">
-        <v>2952.96</v>
+        <v>2896.577</v>
       </c>
       <c r="I46" t="n">
         <v>1422.5</v>
       </c>
       <c r="J46" t="n">
-        <v>3086.0435</v>
+        <v>3019.4167</v>
       </c>
       <c r="K46" t="n">
         <v>1422.5</v>
       </c>
       <c r="L46" t="n">
-        <v>3086.0435</v>
+        <v>3019.4167</v>
       </c>
       <c r="M46" t="n">
         <v>-1234.5</v>
       </c>
       <c r="N46" t="n">
-        <v>-3462.0435</v>
+        <v>-3395.4167</v>
       </c>
     </row>
     <row r="47">
@@ -44854,25 +44842,25 @@
         <v>4333</v>
       </c>
       <c r="H49" t="n">
-        <v>20951</v>
+        <v>40272.555</v>
       </c>
       <c r="I49" t="n">
-        <v>6412.5</v>
+        <v>6262.5</v>
       </c>
       <c r="J49" t="n">
-        <v>50028</v>
+        <v>49989.715</v>
       </c>
       <c r="K49" t="n">
-        <v>6412.5</v>
+        <v>6262.5</v>
       </c>
       <c r="L49" t="n">
-        <v>50028</v>
+        <v>49989.715</v>
       </c>
       <c r="M49" t="n">
-        <v>-6265.5</v>
+        <v>-6115.5</v>
       </c>
       <c r="N49" t="n">
-        <v>-50322</v>
+        <v>-50283.715</v>
       </c>
     </row>
     <row r="50">
@@ -45439,20 +45427,23 @@
         <v>27740</v>
       </c>
       <c r="H61" t="n">
-        <v>35002.5</v>
+        <v>33336.668</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>30005</v>
       </c>
       <c r="J61" t="n">
         <v>35002.5</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>30005</v>
       </c>
       <c r="L61" t="n">
         <v>35002.5</v>
       </c>
+      <c r="M61" t="n">
+        <v>-29803</v>
+      </c>
       <c r="N61" t="n">
         <v>-35406.5</v>
       </c>
@@ -45776,25 +45767,25 @@
         <v>12563</v>
       </c>
       <c r="H68" t="n">
-        <v>3393.7693</v>
+        <v>3710.1667</v>
       </c>
       <c r="I68" t="n">
-        <v>2426.5833</v>
+        <v>2562.9</v>
       </c>
       <c r="J68" t="n">
-        <v>15000</v>
+        <v>9446.5</v>
       </c>
       <c r="K68" t="n">
-        <v>2426.5833</v>
+        <v>2562.9</v>
       </c>
       <c r="L68" t="n">
-        <v>15000</v>
+        <v>9446.5</v>
       </c>
       <c r="M68" t="n">
-        <v>-1677.5833</v>
+        <v>-1813.9</v>
       </c>
       <c r="N68" t="n">
-        <v>-16498</v>
+        <v>-10944.5</v>
       </c>
     </row>
     <row r="69">
@@ -45929,25 +45920,25 @@
         <v>12563</v>
       </c>
       <c r="H71" t="n">
-        <v>3393.7693</v>
+        <v>3710.1667</v>
       </c>
       <c r="I71" t="n">
-        <v>2426.5833</v>
+        <v>2562.9</v>
       </c>
       <c r="J71" t="n">
-        <v>15000</v>
+        <v>9446.5</v>
       </c>
       <c r="K71" t="n">
-        <v>12132.9165</v>
+        <v>12814.5</v>
       </c>
       <c r="L71" t="n">
-        <v>75000</v>
+        <v>47232.5</v>
       </c>
       <c r="M71" t="n">
-        <v>-8388.916499999999</v>
+        <v>-9070.5</v>
       </c>
       <c r="N71" t="n">
-        <v>-82488</v>
+        <v>-54720.5</v>
       </c>
     </row>
     <row r="72">
@@ -46131,22 +46122,25 @@
         <v>10833</v>
       </c>
       <c r="H75" t="n">
-        <v>114999</v>
+        <v>71500</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="J75" t="n">
-        <v>114999</v>
+        <v>113000</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="L75" t="n">
-        <v>114999</v>
+        <v>113000</v>
+      </c>
+      <c r="M75" t="n">
+        <v>-29064</v>
       </c>
       <c r="N75" t="n">
-        <v>-116871</v>
+        <v>-114872</v>
       </c>
     </row>
     <row r="76">
@@ -46278,22 +46272,25 @@
         <v>10833</v>
       </c>
       <c r="H78" t="n">
-        <v>114999</v>
+        <v>71500</v>
       </c>
       <c r="I78" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="J78" t="n">
-        <v>114999</v>
+        <v>113000</v>
       </c>
       <c r="K78" t="n">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="L78" t="n">
-        <v>344997</v>
+        <v>339000</v>
+      </c>
+      <c r="M78" t="n">
+        <v>-85320</v>
       </c>
       <c r="N78" t="n">
-        <v>-354357</v>
+        <v>-348360</v>
       </c>
     </row>
     <row r="79">
@@ -46716,20 +46713,23 @@
         <v>10926</v>
       </c>
       <c r="H87" t="n">
-        <v>100000</v>
+        <v>97500</v>
       </c>
       <c r="I87" t="n">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="J87" t="n">
         <v>100000</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="L87" t="n">
         <v>100000</v>
       </c>
+      <c r="M87" t="n">
+        <v>-88877</v>
+      </c>
       <c r="N87" t="n">
         <v>-102246</v>
       </c>
@@ -46765,22 +46765,22 @@
         <v>10961</v>
       </c>
       <c r="H88" t="n">
-        <v>87026.5</v>
+        <v>97397.60000000001</v>
       </c>
       <c r="I88" t="n">
-        <v>80542.25</v>
+        <v>95666</v>
       </c>
       <c r="J88" t="n">
         <v>99995</v>
       </c>
       <c r="K88" t="n">
-        <v>80542.25</v>
+        <v>95666</v>
       </c>
       <c r="L88" t="n">
         <v>99995</v>
       </c>
       <c r="M88" t="n">
-        <v>-80114.25</v>
+        <v>-95238</v>
       </c>
       <c r="N88" t="n">
         <v>-100851</v>
@@ -46863,20 +46863,23 @@
         <v>10926</v>
       </c>
       <c r="H90" t="n">
-        <v>100000</v>
+        <v>97500</v>
       </c>
       <c r="I90" t="n">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="J90" t="n">
         <v>100000</v>
       </c>
       <c r="K90" t="n">
-        <v>0</v>
+        <v>270000</v>
       </c>
       <c r="L90" t="n">
         <v>300000</v>
       </c>
+      <c r="M90" t="n">
+        <v>-264384</v>
+      </c>
       <c r="N90" t="n">
         <v>-311232</v>
       </c>
@@ -46912,22 +46915,22 @@
         <v>10961</v>
       </c>
       <c r="H91" t="n">
-        <v>87026.5</v>
+        <v>97397.60000000001</v>
       </c>
       <c r="I91" t="n">
-        <v>80542.25</v>
+        <v>95666</v>
       </c>
       <c r="J91" t="n">
         <v>99995</v>
       </c>
       <c r="K91" t="n">
-        <v>80542.25</v>
+        <v>95666</v>
       </c>
       <c r="L91" t="n">
         <v>99995</v>
       </c>
       <c r="M91" t="n">
-        <v>-79060.25</v>
+        <v>-94184</v>
       </c>
       <c r="N91" t="n">
         <v>-102959</v>
@@ -47016,22 +47019,22 @@
         <v>19993</v>
       </c>
       <c r="H93" t="n">
-        <v>72764.62</v>
+        <v>104021.89</v>
       </c>
       <c r="I93" t="n">
-        <v>93094.10000000001</v>
+        <v>153533</v>
       </c>
       <c r="J93" t="n">
         <v>4999.6665</v>
       </c>
       <c r="K93" t="n">
-        <v>93094.10000000001</v>
+        <v>153533</v>
       </c>
       <c r="L93" t="n">
         <v>4999.6665</v>
       </c>
       <c r="M93" t="n">
-        <v>-91846.10000000001</v>
+        <v>-152285</v>
       </c>
       <c r="N93" t="n">
         <v>-7495.6665</v>
@@ -47598,22 +47601,22 @@
         <v>18698</v>
       </c>
       <c r="H105" t="n">
-        <v>120999</v>
+        <v>120993.5</v>
       </c>
       <c r="I105" t="n">
         <v>0</v>
       </c>
       <c r="J105" t="n">
-        <v>120999</v>
+        <v>120993.5</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
       </c>
       <c r="L105" t="n">
-        <v>120999</v>
+        <v>120993.5</v>
       </c>
       <c r="N105" t="n">
-        <v>-127987</v>
+        <v>-127981.5</v>
       </c>
     </row>
     <row r="106">
@@ -47987,20 +47990,23 @@
         <v>27740</v>
       </c>
       <c r="H113" t="n">
-        <v>35002.5</v>
+        <v>33336.668</v>
       </c>
       <c r="I113" t="n">
-        <v>0</v>
+        <v>30005</v>
       </c>
       <c r="J113" t="n">
         <v>35002.5</v>
       </c>
       <c r="K113" t="n">
-        <v>0</v>
+        <v>30005</v>
       </c>
       <c r="L113" t="n">
         <v>35002.5</v>
       </c>
+      <c r="M113" t="n">
+        <v>-27835</v>
+      </c>
       <c r="N113" t="n">
         <v>-39342.5</v>
       </c>
@@ -48428,22 +48434,25 @@
         <v>36247</v>
       </c>
       <c r="H122" t="n">
-        <v>18995</v>
+        <v>12222.75</v>
       </c>
       <c r="I122" t="n">
-        <v>0</v>
+        <v>9966</v>
       </c>
       <c r="J122" t="n">
-        <v>18995</v>
+        <v>18993</v>
       </c>
       <c r="K122" t="n">
-        <v>0</v>
+        <v>29898</v>
       </c>
       <c r="L122" t="n">
-        <v>56985</v>
+        <v>56979</v>
+      </c>
+      <c r="M122" t="n">
+        <v>-27448</v>
       </c>
       <c r="N122" t="n">
-        <v>-61885</v>
+        <v>-61879</v>
       </c>
     </row>
     <row r="123">
@@ -48621,25 +48630,25 @@
         <v>36249</v>
       </c>
       <c r="H126" t="n">
-        <v>6124.875</v>
+        <v>5760.3</v>
       </c>
       <c r="I126" t="n">
-        <v>4599</v>
+        <v>4932.3335</v>
       </c>
       <c r="J126" t="n">
-        <v>8668</v>
+        <v>7002.25</v>
       </c>
       <c r="K126" t="n">
-        <v>13797</v>
+        <v>14797.0005</v>
       </c>
       <c r="L126" t="n">
-        <v>26004</v>
+        <v>21006.75</v>
       </c>
       <c r="M126" t="n">
-        <v>-11327</v>
+        <v>-12327.0005</v>
       </c>
       <c r="N126" t="n">
-        <v>-30944</v>
+        <v>-25946.75</v>
       </c>
     </row>
     <row r="127">
@@ -48915,22 +48924,22 @@
         <v>44058</v>
       </c>
       <c r="H132" t="n">
-        <v>8750.909</v>
+        <v>8887</v>
       </c>
       <c r="I132" t="n">
-        <v>7302.759</v>
+        <v>7406.5713</v>
       </c>
       <c r="J132" t="n">
         <v>19250</v>
       </c>
       <c r="K132" t="n">
-        <v>21908.277</v>
+        <v>22219.7139</v>
       </c>
       <c r="L132" t="n">
         <v>57750</v>
       </c>
       <c r="M132" t="n">
-        <v>-19378.277</v>
+        <v>-19689.7139</v>
       </c>
       <c r="N132" t="n">
         <v>-62810</v>
@@ -49111,22 +49120,22 @@
         <v>44060</v>
       </c>
       <c r="H136" t="n">
-        <v>3371.7307</v>
+        <v>3250.7585</v>
       </c>
       <c r="I136" t="n">
-        <v>3386.6</v>
+        <v>3259.7144</v>
       </c>
       <c r="J136" t="n">
         <v>3000</v>
       </c>
       <c r="K136" t="n">
-        <v>10159.8</v>
+        <v>9779.143199999999</v>
       </c>
       <c r="L136" t="n">
         <v>9000</v>
       </c>
       <c r="M136" t="n">
-        <v>-7609.799999999999</v>
+        <v>-7229.143199999999</v>
       </c>
       <c r="N136" t="n">
         <v>-14100</v>
@@ -50045,25 +50054,25 @@
         <v>3008</v>
       </c>
       <c r="H13" t="n">
-        <v>7727071.5</v>
+        <v>18011334</v>
       </c>
       <c r="I13" t="n">
-        <v>15833.333</v>
+        <v>17000</v>
       </c>
       <c r="J13" t="n">
-        <v>13510500</v>
+        <v>54000000</v>
       </c>
       <c r="K13" t="n">
-        <v>15833.333</v>
+        <v>17000</v>
       </c>
       <c r="L13" t="n">
-        <v>13510500</v>
+        <v>54000000</v>
       </c>
       <c r="M13" t="n">
-        <v>-15693.333</v>
+        <v>-16860</v>
       </c>
       <c r="N13" t="n">
-        <v>-13510780</v>
+        <v>-54000280</v>
       </c>
     </row>
     <row r="14">
@@ -50605,19 +50614,22 @@
         <v>3561</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>26009</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>26009</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>26009</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>-25779</v>
       </c>
     </row>
     <row r="25">
@@ -50847,22 +50859,22 @@
         <v>3568</v>
       </c>
       <c r="H29" t="n">
-        <v>27010</v>
+        <v>30010</v>
       </c>
       <c r="I29" t="n">
-        <v>27010</v>
+        <v>30010</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>27010</v>
+        <v>30010</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>-26720</v>
+        <v>-29720</v>
       </c>
     </row>
     <row r="30">
@@ -51040,22 +51052,22 @@
         <v>2734</v>
       </c>
       <c r="H33" t="n">
-        <v>25042.666</v>
+        <v>25529.5</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>25042.666</v>
+        <v>25529.5</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>25042.666</v>
+        <v>25529.5</v>
       </c>
       <c r="N33" t="n">
-        <v>-25542.666</v>
+        <v>-26029.5</v>
       </c>
     </row>
     <row r="34">
@@ -51187,22 +51199,22 @@
         <v>2734</v>
       </c>
       <c r="H36" t="n">
-        <v>25042.666</v>
+        <v>25529.5</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>25042.666</v>
+        <v>25529.5</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>25042.666</v>
+        <v>25529.5</v>
       </c>
       <c r="N36" t="n">
-        <v>-25542.666</v>
+        <v>-26029.5</v>
       </c>
     </row>
     <row r="37">
@@ -52461,25 +52473,25 @@
         <v>12589</v>
       </c>
       <c r="H62" t="n">
-        <v>4527.6113</v>
+        <v>6086</v>
       </c>
       <c r="I62" t="n">
-        <v>4258.5</v>
+        <v>6041</v>
       </c>
       <c r="J62" t="n">
-        <v>4864</v>
+        <v>6140</v>
       </c>
       <c r="K62" t="n">
-        <v>4258.5</v>
+        <v>6041</v>
       </c>
       <c r="L62" t="n">
-        <v>4864</v>
+        <v>6140</v>
       </c>
       <c r="M62" t="n">
-        <v>-3634.5</v>
+        <v>-5417</v>
       </c>
       <c r="N62" t="n">
-        <v>-6112</v>
+        <v>-7388</v>
       </c>
     </row>
     <row r="63">
@@ -52611,25 +52623,25 @@
         <v>12589</v>
       </c>
       <c r="H65" t="n">
-        <v>4527.6113</v>
+        <v>6086</v>
       </c>
       <c r="I65" t="n">
-        <v>4258.5</v>
+        <v>6041</v>
       </c>
       <c r="J65" t="n">
-        <v>4864</v>
+        <v>6140</v>
       </c>
       <c r="K65" t="n">
-        <v>21292.5</v>
+        <v>30205</v>
       </c>
       <c r="L65" t="n">
-        <v>24320</v>
+        <v>30700</v>
       </c>
       <c r="M65" t="n">
-        <v>-18172.5</v>
+        <v>-27085</v>
       </c>
       <c r="N65" t="n">
-        <v>-30560</v>
+        <v>-36940</v>
       </c>
     </row>
     <row r="66">
@@ -55365,25 +55377,25 @@
         <v>36208</v>
       </c>
       <c r="H122" t="n">
-        <v>55560184</v>
+        <v>55560004</v>
       </c>
       <c r="I122" t="n">
-        <v>71433760</v>
+        <v>58827960</v>
       </c>
       <c r="J122" t="n">
-        <v>2673.5</v>
+        <v>4800</v>
       </c>
       <c r="K122" t="n">
-        <v>214301280</v>
+        <v>176483880</v>
       </c>
       <c r="L122" t="n">
-        <v>8020.5</v>
+        <v>14400</v>
       </c>
       <c r="M122" t="n">
-        <v>-214298830</v>
+        <v>-176481430</v>
       </c>
       <c r="N122" t="n">
-        <v>-12920.5</v>
+        <v>-19300</v>
       </c>
     </row>
     <row r="123">
@@ -55558,25 +55570,25 @@
         <v>36210</v>
       </c>
       <c r="H126" t="n">
-        <v>2136.738</v>
+        <v>3114.68</v>
       </c>
       <c r="I126" t="n">
-        <v>2024.2424</v>
+        <v>3027.611</v>
       </c>
       <c r="J126" t="n">
-        <v>2549.2222</v>
+        <v>3338.5715</v>
       </c>
       <c r="K126" t="n">
-        <v>6072.7272</v>
+        <v>9082.832999999999</v>
       </c>
       <c r="L126" t="n">
-        <v>7647.6666</v>
+        <v>10015.7145</v>
       </c>
       <c r="M126" t="n">
-        <v>-3602.7272</v>
+        <v>-6612.832999999999</v>
       </c>
       <c r="N126" t="n">
-        <v>-12587.6666</v>
+        <v>-14955.7145</v>
       </c>
     </row>
     <row r="127">
@@ -55852,22 +55864,22 @@
         <v>44029</v>
       </c>
       <c r="H132" t="n">
-        <v>2193.3726</v>
+        <v>2076.0544</v>
       </c>
       <c r="I132" t="n">
-        <v>2128.1667</v>
+        <v>2009.0962</v>
       </c>
       <c r="J132" t="n">
         <v>3236.6667</v>
       </c>
       <c r="K132" t="n">
-        <v>6384.500100000001</v>
+        <v>6027.2886</v>
       </c>
       <c r="L132" t="n">
         <v>9710.000100000001</v>
       </c>
       <c r="M132" t="n">
-        <v>-3854.500100000001</v>
+        <v>-3497.2886</v>
       </c>
       <c r="N132" t="n">
         <v>-14770.0001</v>
@@ -56048,22 +56060,22 @@
         <v>44031</v>
       </c>
       <c r="H136" t="n">
-        <v>28376.658</v>
+        <v>27656.54</v>
       </c>
       <c r="I136" t="n">
-        <v>1727.2</v>
+        <v>1680.9032</v>
       </c>
       <c r="J136" t="n">
         <v>128312.125</v>
       </c>
       <c r="K136" t="n">
-        <v>5181.6</v>
+        <v>5042.7096</v>
       </c>
       <c r="L136" t="n">
         <v>384936.375</v>
       </c>
       <c r="M136" t="n">
-        <v>-2631.6</v>
+        <v>-2492.7096</v>
       </c>
       <c r="N136" t="n">
         <v>-390036.375</v>

</xml_diff>